<commit_message>
Update Dashboard financiero Sandra González de la Fuente.xlsx
</commit_message>
<xml_diff>
--- a/Dashboard financiero Sandra González de la Fuente.xlsx
+++ b/Dashboard financiero Sandra González de la Fuente.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sandr\OneDrive\Documentos\EXCEL_Y_FINANZAS\MÁSTER EN DISEÑO DE DASHBOARDS Y ANÁLISIS DE DATOS\MÓDULO 6 TIPOS DE DASHBOARDS Y CASOS PRÁCTICOS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sandr\OneDrive\Documentos\GitHub\Dashboard-financiero-Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2C3651-C012-45A0-A086-9E365D93C074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624AA427-94C4-4898-A9B9-A1AD15E20CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="816" activeTab="1" xr2:uid="{92CC657A-38E7-4A41-B255-05C7AC6466A0}"/>
   </bookViews>
@@ -1250,11 +1250,11 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -4297,7 +4297,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F5014612-C4A0-4CF6-8A40-27AEDB09F189}" type="CELLRANGE">
+                    <a:fld id="{81947DFC-60A5-491D-8900-0E8CBF3300A1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4330,7 +4330,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E633A485-1DDB-4982-B8A5-D23477CB1026}" type="CELLRANGE">
+                    <a:fld id="{C85A963F-377E-44E6-A689-1D1680F6CB02}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4364,7 +4364,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7295B63B-7A78-46D8-A033-4D8BD4E3451C}" type="CELLRANGE">
+                    <a:fld id="{2554464C-7C27-438C-9B61-C5E6AAB1C3F4}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4398,7 +4398,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9A93AB6B-6C17-4629-975D-9F84552C5BC2}" type="CELLRANGE">
+                    <a:fld id="{A70CDDBA-6FDB-4F03-B317-5853B1750590}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4432,7 +4432,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{846A0383-59E6-4D57-A4B1-C89E2C693493}" type="CELLRANGE">
+                    <a:fld id="{BDCFD629-B258-4E63-B353-860A3E0F5DBE}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4466,7 +4466,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E746D045-1CD9-44DC-BCB9-D8A417C3DD0C}" type="CELLRANGE">
+                    <a:fld id="{56A71B0B-A59B-4F99-9529-6A060BE37D92}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4500,7 +4500,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{25DDD58E-0AA1-4028-88F4-F71C2000AB71}" type="CELLRANGE">
+                    <a:fld id="{9931518F-36F2-403E-8C81-B8BAE157EC26}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4534,7 +4534,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1655542E-91D4-419E-B11A-E9D143412742}" type="CELLRANGE">
+                    <a:fld id="{BE7378FD-083A-4B88-A9A4-0326A355FAEA}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4568,7 +4568,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{302DC3D8-8D1D-424E-A1FD-6B38CB25999C}" type="CELLRANGE">
+                    <a:fld id="{44994A2A-6CB2-467E-B23F-8E3220AB2CEE}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4602,7 +4602,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9D320263-86B4-4A0C-ABD5-4982B04D82EE}" type="CELLRANGE">
+                    <a:fld id="{F7A04007-92E7-4F29-9539-93904C3187A2}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4636,7 +4636,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9924A433-8C5D-4CDC-85B9-F51249A562C5}" type="CELLRANGE">
+                    <a:fld id="{F50AC333-348F-4BB4-8A07-37F3E9A01736}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -4670,7 +4670,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CEA4E691-1885-49D9-9F5E-1A161F842825}" type="CELLRANGE">
+                    <a:fld id="{8B16D6CC-8723-440A-AE6B-1DDAF4A3228D}" type="CELLRANGE">
                       <a:rPr lang="es-ES"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5906,7 +5906,7 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>17298.765000000003</c:v>
+                  <c:v>18085.072500000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>4762.3891999999996</c:v>
@@ -5915,31 +5915,31 @@
                   <c:v>8342.25</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4336.71</c:v>
+                  <c:v>4458.3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4700.51</c:v>
+                  <c:v>4744.4399999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5836.95</c:v>
+                  <c:v>6392.85</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6394.32</c:v>
+                  <c:v>6633.36</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6858</c:v>
+                  <c:v>6667.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6633.36</c:v>
+                  <c:v>6879.04</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8064.48</c:v>
+                  <c:v>8368.7999999999993</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8398.08</c:v>
+                  <c:v>8942.4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>8288.0499999999993</c:v>
+                  <c:v>7927.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7032,34 +7032,34 @@
                   <c:v>5389.2793000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4494.1104000000005</c:v>
+                  <c:v>4450.8978000000006</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1780.4580000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3465.4246999999996</c:v>
+                  <c:v>3532.7144999999996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4242.2016000000003</c:v>
+                  <c:v>4201.4111999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6759.4589999999998</c:v>
+                  <c:v>6630.7074000000002</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>5301.5130000000008</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2536.0816</c:v>
+                  <c:v>2560.4670000000001</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>3871.92</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2818.7952</c:v>
+                  <c:v>2791.6914000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1709.5575000000001</c:v>
+                  <c:v>1676.9945</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>3535.5162</c:v>
@@ -8014,40 +8014,40 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>11909.485700000003</c:v>
+                  <c:v>12695.793200000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>268.27879999999914</c:v>
+                  <c:v>311.49139999999898</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>6561.7919999999995</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>871.28530000000046</c:v>
+                  <c:v>925.58550000000059</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>458.30839999999989</c:v>
+                  <c:v>543.02880000000005</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-922.50900000000001</c:v>
+                  <c:v>-237.85739999999987</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1092.8069999999989</c:v>
+                  <c:v>1331.8469999999988</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4321.9184000000005</c:v>
+                  <c:v>4107.0329999999994</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2761.4399999999996</c:v>
+                  <c:v>3007.12</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5245.6847999999991</c:v>
+                  <c:v>5577.1085999999996</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>6688.5225</c:v>
+                  <c:v>7265.4054999999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4752.5337999999992</c:v>
+                  <c:v>4392.1837999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13500,10 +13500,10 @@
       <c r="AR1">
         <v>0</v>
       </c>
-      <c r="AT1" s="128" t="s">
+      <c r="AT1" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="AU1" s="128"/>
+      <c r="AU1" s="129"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A2" s="33">
@@ -13755,7 +13755,7 @@
       </c>
       <c r="AF3" s="93">
         <f ca="1">(RANDBETWEEN($AT$3,$AU$3)*Q3/100)+Q3</f>
-        <v>17298.765000000003</v>
+        <v>18085.072500000002</v>
       </c>
       <c r="AG3" s="93">
         <f t="shared" ref="AG3:AQ3" ca="1" si="0">(RANDBETWEEN($AT$3,$AU$3)*R3/100)+R3</f>
@@ -13767,43 +13767,43 @@
       </c>
       <c r="AI3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>4336.71</v>
+        <v>4458.3</v>
       </c>
       <c r="AJ3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>4700.51</v>
+        <v>4744.4399999999996</v>
       </c>
       <c r="AK3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>5836.95</v>
+        <v>6392.85</v>
       </c>
       <c r="AL3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>6394.32</v>
+        <v>6633.36</v>
       </c>
       <c r="AM3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>6858</v>
+        <v>6667.5</v>
       </c>
       <c r="AN3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>6633.36</v>
+        <v>6879.04</v>
       </c>
       <c r="AO3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8064.48</v>
+        <v>8368.7999999999993</v>
       </c>
       <c r="AP3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8398.08</v>
+        <v>8942.4</v>
       </c>
       <c r="AQ3" s="93">
         <f t="shared" ca="1" si="0"/>
-        <v>8288.0499999999993</v>
+        <v>7927.7</v>
       </c>
       <c r="AR3" s="63">
         <f ca="1">SUM(AF3:AQ3)</f>
-        <v>89913.864200000011</v>
+        <v>92204.101699999999</v>
       </c>
       <c r="AS3" s="53"/>
       <c r="AT3" s="66">
@@ -13845,7 +13845,7 @@
       <c r="AE4" s="8"/>
       <c r="AF4" s="69">
         <f ca="1">AF3/Q3-1</f>
-        <v>9.9999999999999867E-2</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="AG4" s="69">
         <f t="shared" ref="AG4:AR4" ca="1" si="1">AG3/R3-1</f>
@@ -13857,43 +13857,43 @@
       </c>
       <c r="AI4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>7.0000000000000062E-2</v>
+        <v>0.10000000000000009</v>
       </c>
       <c r="AJ4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>7.0000000000000062E-2</v>
+        <v>7.9999999999999849E-2</v>
       </c>
       <c r="AK4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>5.0000000000000044E-2</v>
+        <v>0.15000000000000013</v>
       </c>
       <c r="AL4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>7.0000000000000062E-2</v>
+        <v>0.10999999999999988</v>
       </c>
       <c r="AM4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>8.0000000000000071E-2</v>
+        <v>5.0000000000000044E-2</v>
       </c>
       <c r="AN4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>7.9999999999999849E-2</v>
+        <v>0.11999999999999988</v>
       </c>
       <c r="AO4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>6.0000000000000053E-2</v>
+        <v>9.9999999999999867E-2</v>
       </c>
       <c r="AP4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>8.0000000000000071E-2</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="AQ4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>0.14999999999999991</v>
+        <v>9.9999999999999867E-2</v>
       </c>
       <c r="AR4" s="69">
         <f t="shared" ca="1" si="1"/>
-        <v>8.0332299346001168E-2</v>
+        <v>0.10784994155210081</v>
       </c>
       <c r="AS4" s="53"/>
     </row>
@@ -14026,10 +14026,10 @@
         <f t="shared" ref="AR5" si="2">SUM(AF5:AQ5)</f>
         <v>0</v>
       </c>
-      <c r="AT5" s="128" t="s">
+      <c r="AT5" s="129" t="s">
         <v>35</v>
       </c>
-      <c r="AU5" s="128"/>
+      <c r="AU5" s="129"/>
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
@@ -15967,7 +15967,7 @@
       </c>
       <c r="AG22" s="51">
         <f t="shared" ref="AG22:AQ22" ca="1" si="18">(RANDBETWEEN($AT$7,$AU$7)*R22/100)+R22</f>
-        <v>4494.1104000000005</v>
+        <v>4450.8978000000006</v>
       </c>
       <c r="AH22" s="51">
         <f t="shared" ca="1" si="18"/>
@@ -15975,15 +15975,15 @@
       </c>
       <c r="AI22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>3465.4246999999996</v>
+        <v>3532.7144999999996</v>
       </c>
       <c r="AJ22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>4242.2016000000003</v>
+        <v>4201.4111999999996</v>
       </c>
       <c r="AK22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>6759.4589999999998</v>
+        <v>6630.7074000000002</v>
       </c>
       <c r="AL22" s="51">
         <f t="shared" ca="1" si="18"/>
@@ -15991,7 +15991,7 @@
       </c>
       <c r="AM22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>2536.0816</v>
+        <v>2560.4670000000001</v>
       </c>
       <c r="AN22" s="51">
         <f t="shared" ca="1" si="18"/>
@@ -15999,11 +15999,11 @@
       </c>
       <c r="AO22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>2818.7952</v>
+        <v>2791.6914000000002</v>
       </c>
       <c r="AP22" s="51">
         <f t="shared" ca="1" si="18"/>
-        <v>1709.5575000000001</v>
+        <v>1676.9945</v>
       </c>
       <c r="AQ22" s="51">
         <f t="shared" ca="1" si="18"/>
@@ -16011,7 +16011,7 @@
       </c>
       <c r="AR22" s="52">
         <f ca="1">SUM(AF22:AQ22)</f>
-        <v>45904.316500000001</v>
+        <v>45723.570299999999</v>
       </c>
     </row>
     <row r="23" spans="1:47" x14ac:dyDescent="0.3">
@@ -16130,7 +16130,7 @@
       </c>
       <c r="AF23" s="6">
         <f t="shared" ref="AF23:AQ23" ca="1" si="21">AF3-AF7-AF12</f>
-        <v>17298.765000000003</v>
+        <v>18085.072500000002</v>
       </c>
       <c r="AG23" s="6">
         <f t="shared" ca="1" si="21"/>
@@ -16142,43 +16142,43 @@
       </c>
       <c r="AI23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>4336.71</v>
+        <v>4458.3</v>
       </c>
       <c r="AJ23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>4700.51</v>
+        <v>4744.4399999999996</v>
       </c>
       <c r="AK23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>5836.95</v>
+        <v>6392.85</v>
       </c>
       <c r="AL23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>6394.32</v>
+        <v>6633.36</v>
       </c>
       <c r="AM23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>6858</v>
+        <v>6667.5</v>
       </c>
       <c r="AN23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>6633.36</v>
+        <v>6879.04</v>
       </c>
       <c r="AO23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8064.48</v>
+        <v>8368.7999999999993</v>
       </c>
       <c r="AP23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8398.08</v>
+        <v>8942.4</v>
       </c>
       <c r="AQ23" s="6">
         <f t="shared" ca="1" si="21"/>
-        <v>8288.0499999999993</v>
+        <v>7927.7</v>
       </c>
       <c r="AR23" s="7">
         <f ca="1">SUM(AF23:AQ23)</f>
-        <v>89913.864200000011</v>
+        <v>92204.101699999999</v>
       </c>
     </row>
     <row r="24" spans="1:47" x14ac:dyDescent="0.3">
@@ -16527,11 +16527,11 @@
       </c>
       <c r="AF28" s="32">
         <f ca="1">AF3-AF22</f>
-        <v>11909.485700000003</v>
+        <v>12695.793200000002</v>
       </c>
       <c r="AG28" s="32">
         <f t="shared" ref="AG28:AQ28" ca="1" si="25">AG3-AG22</f>
-        <v>268.27879999999914</v>
+        <v>311.49139999999898</v>
       </c>
       <c r="AH28" s="32">
         <f t="shared" ca="1" si="25"/>
@@ -16539,43 +16539,43 @@
       </c>
       <c r="AI28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>871.28530000000046</v>
+        <v>925.58550000000059</v>
       </c>
       <c r="AJ28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>458.30839999999989</v>
+        <v>543.02880000000005</v>
       </c>
       <c r="AK28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>-922.50900000000001</v>
+        <v>-237.85739999999987</v>
       </c>
       <c r="AL28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>1092.8069999999989</v>
+        <v>1331.8469999999988</v>
       </c>
       <c r="AM28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>4321.9184000000005</v>
+        <v>4107.0329999999994</v>
       </c>
       <c r="AN28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>2761.4399999999996</v>
+        <v>3007.12</v>
       </c>
       <c r="AO28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>5245.6847999999991</v>
+        <v>5577.1085999999996</v>
       </c>
       <c r="AP28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>6688.5225</v>
+        <v>7265.4054999999998</v>
       </c>
       <c r="AQ28" s="32">
         <f t="shared" ca="1" si="25"/>
-        <v>4752.5337999999992</v>
+        <v>4392.1837999999998</v>
       </c>
       <c r="AR28" s="32">
         <f ca="1">SUM(AF28:AQ28)</f>
-        <v>44009.547699999996</v>
+        <v>46480.5314</v>
       </c>
     </row>
     <row r="29" spans="1:47" x14ac:dyDescent="0.3">
@@ -16738,11 +16738,11 @@
       </c>
       <c r="AF30" s="15">
         <f t="shared" ref="AF30:AQ30" ca="1" si="28">AF28</f>
-        <v>11909.485700000003</v>
+        <v>12695.793200000002</v>
       </c>
       <c r="AG30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>268.27879999999914</v>
+        <v>311.49139999999898</v>
       </c>
       <c r="AH30" s="15">
         <f t="shared" ca="1" si="28"/>
@@ -16750,43 +16750,43 @@
       </c>
       <c r="AI30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>871.28530000000046</v>
+        <v>925.58550000000059</v>
       </c>
       <c r="AJ30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>458.30839999999989</v>
+        <v>543.02880000000005</v>
       </c>
       <c r="AK30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>-922.50900000000001</v>
+        <v>-237.85739999999987</v>
       </c>
       <c r="AL30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>1092.8069999999989</v>
+        <v>1331.8469999999988</v>
       </c>
       <c r="AM30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>4321.9184000000005</v>
+        <v>4107.0329999999994</v>
       </c>
       <c r="AN30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>2761.4399999999996</v>
+        <v>3007.12</v>
       </c>
       <c r="AO30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>5245.6847999999991</v>
+        <v>5577.1085999999996</v>
       </c>
       <c r="AP30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>6688.5225</v>
+        <v>7265.4054999999998</v>
       </c>
       <c r="AQ30" s="15">
         <f t="shared" ca="1" si="28"/>
-        <v>4752.5337999999992</v>
+        <v>4392.1837999999998</v>
       </c>
       <c r="AR30" s="15">
         <f ca="1">SUM(AF30:AQ30)</f>
-        <v>44009.547699999996</v>
+        <v>46480.5314</v>
       </c>
     </row>
     <row r="31" spans="1:47" x14ac:dyDescent="0.3">
@@ -16897,11 +16897,11 @@
       <c r="AE31" s="10"/>
       <c r="AF31" s="16">
         <f t="shared" ref="AF31:AR31" ca="1" si="31">AF30/AF3</f>
-        <v>0.68845872523269724</v>
+        <v>0.70200399804866698</v>
       </c>
       <c r="AG31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>5.6332817149845532E-2</v>
+        <v>6.540654006186622E-2</v>
       </c>
       <c r="AH31" s="16">
         <f t="shared" ca="1" si="31"/>
@@ -16909,43 +16909,43 @@
       </c>
       <c r="AI31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.20090928376580414</v>
+        <v>0.20760951483749424</v>
       </c>
       <c r="AJ31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>9.7501845544419624E-2</v>
+        <v>0.11445582618812759</v>
       </c>
       <c r="AK31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>-0.15804641122504048</v>
+        <v>-3.7206785705905791E-2</v>
       </c>
       <c r="AL31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.17090276995833786</v>
+        <v>0.20078014761749685</v>
       </c>
       <c r="AM31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.63020099154272391</v>
+        <v>0.61597795275590539</v>
       </c>
       <c r="AN31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.41629581388617531</v>
+        <v>0.43714239196166904</v>
       </c>
       <c r="AO31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.65046782929587521</v>
+        <v>0.66641676225982216</v>
       </c>
       <c r="AP31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.79643472079332422</v>
+        <v>0.81246706700662019</v>
       </c>
       <c r="AQ31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.57342002039080353</v>
+        <v>0.55403002131765833</v>
       </c>
       <c r="AR31" s="16">
         <f t="shared" ca="1" si="31"/>
-        <v>0.48946342248295888</v>
+        <v>0.50410481250857408</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
@@ -17093,60 +17093,60 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="129" t="str">
+      <c r="A2" s="128" t="str">
         <f>CONCATENATE("Ventas totales", " ", I8)</f>
         <v>Ventas totales Mayo</v>
       </c>
-      <c r="B2" s="129"/>
-      <c r="C2" s="129"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="129"/>
-      <c r="F2" s="129"/>
-      <c r="U2" s="129" t="str">
+      <c r="B2" s="128"/>
+      <c r="C2" s="128"/>
+      <c r="D2" s="128"/>
+      <c r="E2" s="128"/>
+      <c r="F2" s="128"/>
+      <c r="U2" s="128" t="str">
         <f>CONCATENATE("Ventas acumuladas")</f>
         <v>Ventas acumuladas</v>
       </c>
-      <c r="V2" s="129"/>
-      <c r="W2" s="129"/>
-      <c r="X2" s="129"/>
-      <c r="Y2" s="129"/>
-      <c r="Z2" s="129"/>
-      <c r="AA2" s="129"/>
-      <c r="AB2" s="129"/>
+      <c r="V2" s="128"/>
+      <c r="W2" s="128"/>
+      <c r="X2" s="128"/>
+      <c r="Y2" s="128"/>
+      <c r="Z2" s="128"/>
+      <c r="AA2" s="128"/>
+      <c r="AB2" s="128"/>
     </row>
     <row r="3" spans="1:28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="129"/>
-      <c r="B3" s="129"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="129"/>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
+      <c r="A3" s="128"/>
+      <c r="B3" s="128"/>
+      <c r="C3" s="128"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="128"/>
       <c r="G3" s="98"/>
-      <c r="U3" s="129"/>
-      <c r="V3" s="129"/>
-      <c r="W3" s="129"/>
-      <c r="X3" s="129"/>
-      <c r="Y3" s="129"/>
-      <c r="Z3" s="129"/>
-      <c r="AA3" s="129"/>
-      <c r="AB3" s="129"/>
+      <c r="U3" s="128"/>
+      <c r="V3" s="128"/>
+      <c r="W3" s="128"/>
+      <c r="X3" s="128"/>
+      <c r="Y3" s="128"/>
+      <c r="Z3" s="128"/>
+      <c r="AA3" s="128"/>
+      <c r="AB3" s="128"/>
     </row>
     <row r="4" spans="1:28" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="129"/>
-      <c r="B4" s="129"/>
-      <c r="C4" s="129"/>
-      <c r="D4" s="129"/>
-      <c r="E4" s="129"/>
-      <c r="F4" s="129"/>
+      <c r="A4" s="128"/>
+      <c r="B4" s="128"/>
+      <c r="C4" s="128"/>
+      <c r="D4" s="128"/>
+      <c r="E4" s="128"/>
+      <c r="F4" s="128"/>
       <c r="G4" s="98"/>
-      <c r="U4" s="129"/>
-      <c r="V4" s="129"/>
-      <c r="W4" s="129"/>
-      <c r="X4" s="129"/>
-      <c r="Y4" s="129"/>
-      <c r="Z4" s="129"/>
-      <c r="AA4" s="129"/>
-      <c r="AB4" s="129"/>
+      <c r="U4" s="128"/>
+      <c r="V4" s="128"/>
+      <c r="W4" s="128"/>
+      <c r="X4" s="128"/>
+      <c r="Y4" s="128"/>
+      <c r="Z4" s="128"/>
+      <c r="AA4" s="128"/>
+      <c r="AB4" s="128"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="N5" s="126"/>
@@ -17228,19 +17228,19 @@
       </c>
       <c r="Q9" s="114">
         <f ca="1">VLOOKUP(H9,'Cta Resultados'!$AE$3:$AR$30,MATCH('Mi dashboard'!$I$8,'Cta Resultados'!$AE$2:$AR$2,0),0)</f>
-        <v>4700.51</v>
+        <v>4744.4399999999996</v>
       </c>
       <c r="R9" s="111">
         <f ca="1">IFERROR(I9/Q9-1,"")</f>
-        <v>-0.13775313742551343</v>
+        <v>-0.14573690467157341</v>
       </c>
       <c r="S9" s="122">
         <f ca="1">SUMPRODUCT('Cta Resultados'!AF3:AQ3,'Cta Resultados'!AF1:AQ1)</f>
-        <v>58529.894200000002</v>
+        <v>60086.161700000004</v>
       </c>
       <c r="T9" s="113">
         <f ca="1">IFERROR(I9/S9-1,"")</f>
-        <v>-0.93075333459256449</v>
+        <v>-0.93254686461358705</v>
       </c>
     </row>
     <row r="10" spans="1:28" ht="21" x14ac:dyDescent="0.4">
@@ -17468,19 +17468,19 @@
       <c r="P17" s="109"/>
       <c r="Q17" s="117">
         <f ca="1">VLOOKUP('Cta Resultados'!AE30,'Cta Resultados'!$AE$3:$AR$30,MATCH('Mi dashboard'!$I$8,'Cta Resultados'!$AE$2:$AR$2,0),0)</f>
-        <v>458.30839999999989</v>
+        <v>543.02880000000005</v>
       </c>
       <c r="R17" s="119">
         <f ca="1">IFERROR(I17/Q17-1,"")</f>
-        <v>0.5022853606872586</v>
+        <v>0.26790696920679014</v>
       </c>
       <c r="S17" s="123">
         <f ca="1">SUMPRODUCT('Cta Resultados'!AF30:AQ30,'Cta Resultados'!AF1:AQ1)</f>
-        <v>24561.366600000001</v>
+        <v>26238.713499999998</v>
       </c>
       <c r="T17" s="119">
         <f ca="1">IFERROR(I17/S17-1,"")</f>
-        <v>-0.9719677650184172</v>
+        <v>-0.9737597653177622</v>
       </c>
       <c r="U17" s="109"/>
     </row>

</xml_diff>